<commit_message>
Verify masked fixtures retain observed text percentage and numeric column types
</commit_message>
<xml_diff>
--- a/staging/imile-management/reports/fixtures/MASKED_ofd.xlsx
+++ b/staging/imile-management/reports/fixtures/MASKED_ofd.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R35cadf18074b4547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rce91361ecc7441d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -442,8 +442,8 @@
       <x:c r="K2" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L2" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="L2" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="M2" s="4" t="n">
         <x:v>0</x:v>
@@ -463,14 +463,14 @@
       <x:c r="R2" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U2" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="S2" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="T2" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="U2" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="V2" s="4" t="n">
         <x:v>0</x:v>
@@ -478,8 +478,8 @@
       <x:c r="W2" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="X2" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="X2" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="Y2" s="4" t="n">
         <x:v>0</x:v>
@@ -493,17 +493,17 @@
       <x:c r="AB2" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AC2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AE2" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AF2" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="AC2" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AD2" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AE2" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AF2" s="4" t="str">
+        <x:v>MASKED</x:v>
       </x:c>
       <x:c r="AG2" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
@@ -549,8 +549,8 @@
       <x:c r="K3" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L3" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="L3" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="M3" s="4" t="n">
         <x:v>0</x:v>
@@ -570,14 +570,14 @@
       <x:c r="R3" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U3" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="S3" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="T3" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="U3" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="V3" s="4" t="n">
         <x:v>0</x:v>
@@ -585,8 +585,8 @@
       <x:c r="W3" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="X3" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="X3" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="Y3" s="4" t="n">
         <x:v>0</x:v>
@@ -600,17 +600,17 @@
       <x:c r="AB3" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AC3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AE3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AF3" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="AC3" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AD3" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AE3" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AF3" s="4" t="str">
+        <x:v>MASKED</x:v>
       </x:c>
       <x:c r="AG3" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
@@ -656,8 +656,8 @@
       <x:c r="K4" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L4" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="L4" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="M4" s="4" t="n">
         <x:v>0</x:v>
@@ -677,14 +677,14 @@
       <x:c r="R4" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U4" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="S4" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="T4" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="U4" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="V4" s="4" t="n">
         <x:v>0</x:v>
@@ -692,8 +692,8 @@
       <x:c r="W4" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="X4" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="X4" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="Y4" s="4" t="n">
         <x:v>0</x:v>
@@ -707,17 +707,17 @@
       <x:c r="AB4" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AC4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AE4" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AF4" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="AC4" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AD4" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AE4" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AF4" s="4" t="str">
+        <x:v>MASKED</x:v>
       </x:c>
       <x:c r="AG4" s="3" t="str">
         <x:v>DS(SYN_AKE)</x:v>
@@ -763,8 +763,8 @@
       <x:c r="K5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="L5" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="M5" s="4" t="n">
         <x:v>0</x:v>
@@ -784,14 +784,14 @@
       <x:c r="R5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U5" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="S5" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="T5" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="U5" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="V5" s="4" t="n">
         <x:v>0</x:v>
@@ -799,8 +799,8 @@
       <x:c r="W5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="X5" s="3" t="n">
-        <x:v>0</x:v>
+      <x:c r="X5" s="3" t="str">
+        <x:v>0.00%</x:v>
       </x:c>
       <x:c r="Y5" s="4" t="n">
         <x:v>0</x:v>
@@ -814,17 +814,17 @@
       <x:c r="AB5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AC5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AD5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AE5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AF5" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="AC5" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AD5" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AE5" s="3" t="str">
+        <x:v>0.00%</x:v>
+      </x:c>
+      <x:c r="AF5" s="4" t="str">
+        <x:v>MASKED</x:v>
       </x:c>
       <x:c r="AG5" s="3" t="str">
         <x:v>DS(SYN_IKA)</x:v>

</xml_diff>